<commit_message>
Update prim structure with old version
</commit_message>
<xml_diff>
--- a/src/workflow/4_PRIM/prim_files_creator_cntrl.xlsx
+++ b/src/workflow/4_PRIM/prim_files_creator_cntrl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\AFR_RDM\src\workflow\4_PRIM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F27A9C-1648-4F6B-9605-8A0C39DB1501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199EB5C5-944C-4244-B26E-5FD81BB9180B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="match_exp_ana" sheetId="5" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="120">
   <si>
     <t>YES</t>
   </si>
@@ -98,6 +98,15 @@
     <t>Future.ID</t>
   </si>
   <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
     <t>str</t>
   </si>
   <si>
@@ -195,6 +204,189 @@
   </si>
   <si>
     <t>X and L</t>
+  </si>
+  <si>
+    <t>TEM output</t>
+  </si>
+  <si>
+    <t>Fuel_Surname</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Actor</t>
+  </si>
+  <si>
+    <t>Actor_Type</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>GorS</t>
+  </si>
+  <si>
+    <t>DAI</t>
+  </si>
+  <si>
+    <t>Customs</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>VAT-Imports</t>
+  </si>
+  <si>
+    <t>Total Import Taxes</t>
+  </si>
+  <si>
+    <t>GE</t>
+  </si>
+  <si>
+    <t>Vehicle Purchase</t>
+  </si>
+  <si>
+    <t>Property Tax</t>
+  </si>
+  <si>
+    <t>IUC</t>
+  </si>
+  <si>
+    <t>VAT-Electricity</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>VKT</t>
+  </si>
+  <si>
+    <t>Energy Sales and Purchases</t>
+  </si>
+  <si>
+    <t>Investments and FOM</t>
+  </si>
+  <si>
+    <t>Variable Costs</t>
+  </si>
+  <si>
+    <t>Service Sales</t>
+  </si>
+  <si>
+    <t>Service Purchases</t>
+  </si>
+  <si>
+    <t>Investments</t>
+  </si>
+  <si>
+    <t>FOM</t>
+  </si>
+  <si>
+    <t>DAI Disc</t>
+  </si>
+  <si>
+    <t>Customs Disc</t>
+  </si>
+  <si>
+    <t>SC Disc</t>
+  </si>
+  <si>
+    <t>VAT-Imports Disc</t>
+  </si>
+  <si>
+    <t>Total Import Taxes Disc</t>
+  </si>
+  <si>
+    <t>GE Disc</t>
+  </si>
+  <si>
+    <t>Vehicle Purchase Disc</t>
+  </si>
+  <si>
+    <t>Property Tax Disc</t>
+  </si>
+  <si>
+    <t>IUC Disc</t>
+  </si>
+  <si>
+    <t>VAT-Electricity Disc</t>
+  </si>
+  <si>
+    <t>H2 Disc</t>
+  </si>
+  <si>
+    <t>VKT Disc</t>
+  </si>
+  <si>
+    <t>Energy Sales and Purchases Disc</t>
+  </si>
+  <si>
+    <t>Investments and FOM Disc</t>
+  </si>
+  <si>
+    <t>Variable Costs Disc</t>
+  </si>
+  <si>
+    <t>Service Sales Disc</t>
+  </si>
+  <si>
+    <t>Service Purchases Disc</t>
+  </si>
+  <si>
+    <t>Investments Disc</t>
+  </si>
+  <si>
+    <t>FOM Disc</t>
+  </si>
+  <si>
+    <t>Energy Price</t>
+  </si>
+  <si>
+    <t>Energy Price wTax</t>
+  </si>
+  <si>
+    <t>Energy Tax</t>
+  </si>
+  <si>
+    <t>Service Price</t>
+  </si>
+  <si>
+    <t>U SC</t>
+  </si>
+  <si>
+    <t>U Total Import Taxes</t>
+  </si>
+  <si>
+    <t>U Market Price</t>
+  </si>
+  <si>
+    <t>U CIF</t>
+  </si>
+  <si>
+    <t>Q Imports</t>
+  </si>
+  <si>
+    <t>U VKT</t>
+  </si>
+  <si>
+    <t>Q Total</t>
+  </si>
+  <si>
+    <t>U Property Tax</t>
+  </si>
+  <si>
+    <t>FV</t>
+  </si>
+  <si>
+    <t>TEM region</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Gini_Expense</t>
   </si>
   <si>
     <t>Uganda multisectorial model.</t>
@@ -489,7 +681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -532,7 +724,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,27 +1020,27 @@
         <v>1</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="15" t="s">
         <v>41</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>45</v>
+        <v>109</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>0</v>
@@ -858,7 +1049,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>0</v>
@@ -894,7 +1085,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>117</v>
       </c>
       <c r="B2" s="23">
         <v>2021</v>
@@ -905,7 +1096,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B3" s="23">
         <v>2031</v>
@@ -916,7 +1107,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B4" s="23">
         <v>2041</v>
@@ -944,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60477372-007B-42DB-8434-89BB151CD17B}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C164"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -964,409 +1155,1795 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>12</v>
+      <c r="A25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>11</v>
+        <v>48</v>
+      </c>
+      <c r="B26" t="s">
+        <v>68</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>69</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>48</v>
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>70</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>50</v>
+        <v>48</v>
+      </c>
+      <c r="B29" t="s">
+        <v>71</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>31</v>
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>73</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>32</v>
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>74</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>33</v>
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>34</v>
+        <v>48</v>
+      </c>
+      <c r="B34" t="s">
+        <v>76</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" s="24" t="s">
-        <v>35</v>
+        <v>48</v>
+      </c>
+      <c r="B35" t="s">
+        <v>77</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>36</v>
+        <v>48</v>
+      </c>
+      <c r="B36" t="s">
+        <v>78</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B37" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>81</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>91</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" t="s">
+        <v>94</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" t="s">
+        <v>97</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B56" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B58" t="s">
+        <v>100</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B59" t="s">
+        <v>101</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B60" t="s">
+        <v>102</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B61" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B62" t="s">
+        <v>104</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B65" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B67" t="s">
+        <v>113</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B68" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B69" t="s">
+        <v>114</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B70" t="s">
+        <v>115</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B71" t="s">
+        <v>119</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B72" t="s">
+        <v>19</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B73" t="s">
+        <v>20</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B74" t="s">
+        <v>21</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B75" t="s">
+        <v>22</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B76" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B77" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" t="s">
+        <v>25</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" t="s">
+        <v>26</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B80" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" t="s">
+        <v>28</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82" t="s">
+        <v>29</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B83" t="s">
+        <v>30</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B84" t="s">
+        <v>31</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" t="s">
+        <v>32</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" t="s">
+        <v>33</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B88" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B89" t="s">
+        <v>113</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B90" t="s">
+        <v>112</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B91" t="s">
+        <v>114</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" t="s">
+        <v>115</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B93" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B94" t="s">
+        <v>35</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B95" t="s">
+        <v>36</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B96" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C96" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B97" t="s">
+        <v>38</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B98" t="s">
+        <v>39</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B99" t="s">
+        <v>40</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B100" t="s">
+        <v>118</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B102" t="s">
+        <v>11</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B103" t="s">
+        <v>12</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B105" t="s">
+        <v>49</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B106" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" s="9" t="s">
+      <c r="C106" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>50</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B108" t="s">
+        <v>51</v>
+      </c>
+      <c r="C108" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B109" t="s">
+        <v>52</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B110" t="s">
+        <v>53</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B111" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="10" t="s">
-        <v>14</v>
+      <c r="C111" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B112" t="s">
+        <v>55</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B113" t="s">
+        <v>56</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B114" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B115" t="s">
+        <v>58</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B116" t="s">
+        <v>59</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B117" t="s">
+        <v>60</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B118" t="s">
+        <v>61</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B119" t="s">
+        <v>62</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B120" t="s">
+        <v>63</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B121" t="s">
+        <v>64</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B122" t="s">
+        <v>65</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B123" t="s">
+        <v>66</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B124" t="s">
+        <v>67</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B125" t="s">
+        <v>68</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B126" t="s">
+        <v>69</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B127" t="s">
+        <v>70</v>
+      </c>
+      <c r="C127" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B128" t="s">
+        <v>71</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B129" t="s">
+        <v>72</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B130" t="s">
+        <v>73</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B131" t="s">
+        <v>74</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B132" t="s">
+        <v>75</v>
+      </c>
+      <c r="C132" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B133" t="s">
+        <v>76</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B134" t="s">
+        <v>77</v>
+      </c>
+      <c r="C134" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B135" t="s">
+        <v>78</v>
+      </c>
+      <c r="C135" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B136" t="s">
+        <v>79</v>
+      </c>
+      <c r="C136" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B137" t="s">
+        <v>80</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B138" t="s">
+        <v>81</v>
+      </c>
+      <c r="C138" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B139" t="s">
+        <v>82</v>
+      </c>
+      <c r="C139" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B140" t="s">
+        <v>83</v>
+      </c>
+      <c r="C140" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B141" t="s">
+        <v>84</v>
+      </c>
+      <c r="C141" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B142" t="s">
+        <v>85</v>
+      </c>
+      <c r="C142" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B143" t="s">
+        <v>86</v>
+      </c>
+      <c r="C143" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B144" t="s">
+        <v>87</v>
+      </c>
+      <c r="C144" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B145" t="s">
+        <v>88</v>
+      </c>
+      <c r="C145" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B146" t="s">
+        <v>89</v>
+      </c>
+      <c r="C146" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B147" t="s">
+        <v>90</v>
+      </c>
+      <c r="C147" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B148" t="s">
+        <v>91</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B149" t="s">
+        <v>92</v>
+      </c>
+      <c r="C149" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B150" t="s">
+        <v>93</v>
+      </c>
+      <c r="C150" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B151" t="s">
+        <v>94</v>
+      </c>
+      <c r="C151" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B152" t="s">
+        <v>95</v>
+      </c>
+      <c r="C152" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B153" t="s">
+        <v>96</v>
+      </c>
+      <c r="C153" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B154" t="s">
+        <v>97</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B155" t="s">
+        <v>98</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B156" t="s">
+        <v>99</v>
+      </c>
+      <c r="C156" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B157" t="s">
+        <v>100</v>
+      </c>
+      <c r="C157" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B158" t="s">
+        <v>101</v>
+      </c>
+      <c r="C158" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B159" t="s">
+        <v>102</v>
+      </c>
+      <c r="C159" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B160" t="s">
+        <v>103</v>
+      </c>
+      <c r="C160" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B161" t="s">
+        <v>104</v>
+      </c>
+      <c r="C161" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B162" t="s">
+        <v>105</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B163" t="s">
+        <v>107</v>
+      </c>
+      <c r="C163" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C164" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1566,15 +3143,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d55314f-45f1-40c9-9fce-63556e193d03">
@@ -1582,6 +3150,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1603,14 +3180,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC59A38-DB2E-4FA2-8576-7C42CC1FB709}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20E92FB-5FDC-4CBD-AA6F-5B52A6009ECF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1618,4 +3187,12 @@
     <ds:schemaRef ds:uri="0d55314f-45f1-40c9-9fce-63556e193d03"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC59A38-DB2E-4FA2-8576-7C42CC1FB709}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update config files .xlsx of PRIM module to make a test
</commit_message>
<xml_diff>
--- a/src/workflow/4_PRIM/prim_files_creator_cntrl.xlsx
+++ b/src/workflow/4_PRIM/prim_files_creator_cntrl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\AFR_RDM\src\workflow\4_PRIM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12F27A9C-1648-4F6B-9605-8A0C39DB1501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199EB5C5-944C-4244-B26E-5FD81BB9180B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="match_exp_ana" sheetId="5" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="120">
   <si>
     <t>YES</t>
   </si>
@@ -98,6 +98,15 @@
     <t>Future.ID</t>
   </si>
   <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
     <t>str</t>
   </si>
   <si>
@@ -195,6 +204,189 @@
   </si>
   <si>
     <t>X and L</t>
+  </si>
+  <si>
+    <t>TEM output</t>
+  </si>
+  <si>
+    <t>Fuel_Surname</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Actor</t>
+  </si>
+  <si>
+    <t>Actor_Type</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>GorS</t>
+  </si>
+  <si>
+    <t>DAI</t>
+  </si>
+  <si>
+    <t>Customs</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>VAT-Imports</t>
+  </si>
+  <si>
+    <t>Total Import Taxes</t>
+  </si>
+  <si>
+    <t>GE</t>
+  </si>
+  <si>
+    <t>Vehicle Purchase</t>
+  </si>
+  <si>
+    <t>Property Tax</t>
+  </si>
+  <si>
+    <t>IUC</t>
+  </si>
+  <si>
+    <t>VAT-Electricity</t>
+  </si>
+  <si>
+    <t>H2</t>
+  </si>
+  <si>
+    <t>VKT</t>
+  </si>
+  <si>
+    <t>Energy Sales and Purchases</t>
+  </si>
+  <si>
+    <t>Investments and FOM</t>
+  </si>
+  <si>
+    <t>Variable Costs</t>
+  </si>
+  <si>
+    <t>Service Sales</t>
+  </si>
+  <si>
+    <t>Service Purchases</t>
+  </si>
+  <si>
+    <t>Investments</t>
+  </si>
+  <si>
+    <t>FOM</t>
+  </si>
+  <si>
+    <t>DAI Disc</t>
+  </si>
+  <si>
+    <t>Customs Disc</t>
+  </si>
+  <si>
+    <t>SC Disc</t>
+  </si>
+  <si>
+    <t>VAT-Imports Disc</t>
+  </si>
+  <si>
+    <t>Total Import Taxes Disc</t>
+  </si>
+  <si>
+    <t>GE Disc</t>
+  </si>
+  <si>
+    <t>Vehicle Purchase Disc</t>
+  </si>
+  <si>
+    <t>Property Tax Disc</t>
+  </si>
+  <si>
+    <t>IUC Disc</t>
+  </si>
+  <si>
+    <t>VAT-Electricity Disc</t>
+  </si>
+  <si>
+    <t>H2 Disc</t>
+  </si>
+  <si>
+    <t>VKT Disc</t>
+  </si>
+  <si>
+    <t>Energy Sales and Purchases Disc</t>
+  </si>
+  <si>
+    <t>Investments and FOM Disc</t>
+  </si>
+  <si>
+    <t>Variable Costs Disc</t>
+  </si>
+  <si>
+    <t>Service Sales Disc</t>
+  </si>
+  <si>
+    <t>Service Purchases Disc</t>
+  </si>
+  <si>
+    <t>Investments Disc</t>
+  </si>
+  <si>
+    <t>FOM Disc</t>
+  </si>
+  <si>
+    <t>Energy Price</t>
+  </si>
+  <si>
+    <t>Energy Price wTax</t>
+  </si>
+  <si>
+    <t>Energy Tax</t>
+  </si>
+  <si>
+    <t>Service Price</t>
+  </si>
+  <si>
+    <t>U SC</t>
+  </si>
+  <si>
+    <t>U Total Import Taxes</t>
+  </si>
+  <si>
+    <t>U Market Price</t>
+  </si>
+  <si>
+    <t>U CIF</t>
+  </si>
+  <si>
+    <t>Q Imports</t>
+  </si>
+  <si>
+    <t>U VKT</t>
+  </si>
+  <si>
+    <t>Q Total</t>
+  </si>
+  <si>
+    <t>U Property Tax</t>
+  </si>
+  <si>
+    <t>FV</t>
+  </si>
+  <si>
+    <t>TEM region</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Gini_Expense</t>
   </si>
   <si>
     <t>Uganda multisectorial model.</t>
@@ -489,7 +681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -532,7 +724,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,27 +1020,27 @@
         <v>1</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="15" t="s">
         <v>41</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>45</v>
+        <v>109</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>0</v>
@@ -858,7 +1049,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>0</v>
@@ -894,7 +1085,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>117</v>
       </c>
       <c r="B2" s="23">
         <v>2021</v>
@@ -905,7 +1096,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B3" s="23">
         <v>2031</v>
@@ -916,7 +1107,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B4" s="23">
         <v>2041</v>
@@ -944,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60477372-007B-42DB-8434-89BB151CD17B}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C164"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -964,409 +1155,1795 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>12</v>
+      <c r="A25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>11</v>
+        <v>48</v>
+      </c>
+      <c r="B26" t="s">
+        <v>68</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>69</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>48</v>
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>70</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>50</v>
+        <v>48</v>
+      </c>
+      <c r="B29" t="s">
+        <v>71</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>31</v>
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>73</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>32</v>
+        <v>48</v>
+      </c>
+      <c r="B32" t="s">
+        <v>74</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>33</v>
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>34</v>
+        <v>48</v>
+      </c>
+      <c r="B34" t="s">
+        <v>76</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" s="24" t="s">
-        <v>35</v>
+        <v>48</v>
+      </c>
+      <c r="B35" t="s">
+        <v>77</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>36</v>
+        <v>48</v>
+      </c>
+      <c r="B36" t="s">
+        <v>78</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B37" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>81</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>91</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>92</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" t="s">
+        <v>93</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" t="s">
+        <v>94</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" t="s">
+        <v>97</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B56" t="s">
+        <v>98</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" t="s">
+        <v>99</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B58" t="s">
+        <v>100</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B59" t="s">
+        <v>101</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B60" t="s">
+        <v>102</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B61" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B62" t="s">
+        <v>104</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B65" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B67" t="s">
+        <v>113</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B68" t="s">
+        <v>112</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B69" t="s">
+        <v>114</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B70" t="s">
+        <v>115</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B71" t="s">
+        <v>119</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B72" t="s">
+        <v>19</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B73" t="s">
+        <v>20</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B74" t="s">
+        <v>21</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B75" t="s">
+        <v>22</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B76" t="s">
+        <v>23</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B77" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" t="s">
+        <v>25</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" t="s">
+        <v>26</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B80" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" t="s">
+        <v>28</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82" t="s">
+        <v>29</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B83" t="s">
+        <v>30</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B84" t="s">
+        <v>31</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B85" t="s">
+        <v>32</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" t="s">
+        <v>33</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B88" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B89" t="s">
+        <v>113</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B90" t="s">
+        <v>112</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B91" t="s">
+        <v>114</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" t="s">
+        <v>115</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B93" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B94" t="s">
+        <v>35</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B95" t="s">
+        <v>36</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B96" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C96" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B97" t="s">
+        <v>38</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B98" t="s">
+        <v>39</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B99" t="s">
+        <v>40</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B100" t="s">
+        <v>118</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B102" t="s">
+        <v>11</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B103" t="s">
+        <v>12</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B105" t="s">
+        <v>49</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B106" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" s="9" t="s">
+      <c r="C106" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>50</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B108" t="s">
+        <v>51</v>
+      </c>
+      <c r="C108" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B109" t="s">
+        <v>52</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B110" t="s">
+        <v>53</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B111" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="10" t="s">
-        <v>14</v>
+      <c r="C111" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B112" t="s">
+        <v>55</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B113" t="s">
+        <v>56</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B114" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B115" t="s">
+        <v>58</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B116" t="s">
+        <v>59</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B117" t="s">
+        <v>60</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B118" t="s">
+        <v>61</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B119" t="s">
+        <v>62</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B120" t="s">
+        <v>63</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B121" t="s">
+        <v>64</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B122" t="s">
+        <v>65</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B123" t="s">
+        <v>66</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B124" t="s">
+        <v>67</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B125" t="s">
+        <v>68</v>
+      </c>
+      <c r="C125" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B126" t="s">
+        <v>69</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B127" t="s">
+        <v>70</v>
+      </c>
+      <c r="C127" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B128" t="s">
+        <v>71</v>
+      </c>
+      <c r="C128" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B129" t="s">
+        <v>72</v>
+      </c>
+      <c r="C129" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B130" t="s">
+        <v>73</v>
+      </c>
+      <c r="C130" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B131" t="s">
+        <v>74</v>
+      </c>
+      <c r="C131" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B132" t="s">
+        <v>75</v>
+      </c>
+      <c r="C132" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B133" t="s">
+        <v>76</v>
+      </c>
+      <c r="C133" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B134" t="s">
+        <v>77</v>
+      </c>
+      <c r="C134" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B135" t="s">
+        <v>78</v>
+      </c>
+      <c r="C135" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B136" t="s">
+        <v>79</v>
+      </c>
+      <c r="C136" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B137" t="s">
+        <v>80</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B138" t="s">
+        <v>81</v>
+      </c>
+      <c r="C138" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B139" t="s">
+        <v>82</v>
+      </c>
+      <c r="C139" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B140" t="s">
+        <v>83</v>
+      </c>
+      <c r="C140" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B141" t="s">
+        <v>84</v>
+      </c>
+      <c r="C141" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B142" t="s">
+        <v>85</v>
+      </c>
+      <c r="C142" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B143" t="s">
+        <v>86</v>
+      </c>
+      <c r="C143" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B144" t="s">
+        <v>87</v>
+      </c>
+      <c r="C144" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B145" t="s">
+        <v>88</v>
+      </c>
+      <c r="C145" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B146" t="s">
+        <v>89</v>
+      </c>
+      <c r="C146" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B147" t="s">
+        <v>90</v>
+      </c>
+      <c r="C147" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B148" t="s">
+        <v>91</v>
+      </c>
+      <c r="C148" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B149" t="s">
+        <v>92</v>
+      </c>
+      <c r="C149" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B150" t="s">
+        <v>93</v>
+      </c>
+      <c r="C150" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B151" t="s">
+        <v>94</v>
+      </c>
+      <c r="C151" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B152" t="s">
+        <v>95</v>
+      </c>
+      <c r="C152" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B153" t="s">
+        <v>96</v>
+      </c>
+      <c r="C153" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B154" t="s">
+        <v>97</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B155" t="s">
+        <v>98</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B156" t="s">
+        <v>99</v>
+      </c>
+      <c r="C156" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B157" t="s">
+        <v>100</v>
+      </c>
+      <c r="C157" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B158" t="s">
+        <v>101</v>
+      </c>
+      <c r="C158" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B159" t="s">
+        <v>102</v>
+      </c>
+      <c r="C159" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B160" t="s">
+        <v>103</v>
+      </c>
+      <c r="C160" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B161" t="s">
+        <v>104</v>
+      </c>
+      <c r="C161" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B162" t="s">
+        <v>105</v>
+      </c>
+      <c r="C162" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B163" t="s">
+        <v>107</v>
+      </c>
+      <c r="C163" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C164" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1566,15 +3143,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d55314f-45f1-40c9-9fce-63556e193d03">
@@ -1582,6 +3150,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1603,14 +3180,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC59A38-DB2E-4FA2-8576-7C42CC1FB709}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F20E92FB-5FDC-4CBD-AA6F-5B52A6009ECF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1618,4 +3187,12 @@
     <ds:schemaRef ds:uri="0d55314f-45f1-40c9-9fce-63556e193d03"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CC59A38-DB2E-4FA2-8576-7C42CC1FB709}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>